<commit_message>
Update to New Branch
</commit_message>
<xml_diff>
--- a/outputs/question_bank_sample_pasted_questions.xlsx
+++ b/outputs/question_bank_sample_pasted_questions.xlsx
@@ -68,12 +68,12 @@
     <col min="2" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="24" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="58" customWidth="1"/>
-    <col min="7" max="7" width="38" customWidth="1"/>
-    <col min="8" max="8" width="66" customWidth="1"/>
-    <col min="9" max="9" width="32" customWidth="1"/>
-    <col min="10" max="10" width="16" customWidth="1"/>
+    <col min="5" max="5" width="58" customWidth="1"/>
+    <col min="6" max="6" width="38" customWidth="1"/>
+    <col min="7" max="7" width="66" customWidth="1"/>
+    <col min="8" max="8" width="32" customWidth="1"/>
+    <col min="9" max="9" width="16" customWidth="1"/>
+    <col min="10" max="10" width="24" customWidth="1"/>
     <col min="11" max="11" width="24" customWidth="1"/>
     <col min="12" max="12" width="24" customWidth="1"/>
     <col min="13" max="13" width="24" customWidth="1"/>
@@ -83,16 +83,17 @@
     <col min="17" max="17" width="24" customWidth="1"/>
     <col min="18" max="18" width="24" customWidth="1"/>
     <col min="19" max="19" width="24" customWidth="1"/>
-    <col min="20" max="20" width="24" customWidth="1"/>
-    <col min="21" max="21" width="16" customWidth="1"/>
-    <col min="22" max="22" width="58" customWidth="1"/>
-    <col min="23" max="23" width="14" customWidth="1"/>
-    <col min="24" max="24" width="10" customWidth="1"/>
-    <col min="25" max="25" width="14" customWidth="1"/>
-    <col min="26" max="26" width="10" customWidth="1"/>
-    <col min="27" max="27" width="16" customWidth="1"/>
+    <col min="20" max="20" width="16" customWidth="1"/>
+    <col min="21" max="21" width="58" customWidth="1"/>
+    <col min="22" max="22" width="14" customWidth="1"/>
+    <col min="23" max="23" width="10" customWidth="1"/>
+    <col min="24" max="24" width="14" customWidth="1"/>
+    <col min="25" max="25" width="10" customWidth="1"/>
+    <col min="26" max="26" width="16" customWidth="1"/>
+    <col min="27" max="27" width="18" customWidth="1"/>
     <col min="28" max="28" width="16" customWidth="1"/>
-    <col min="29" max="29" width="58" customWidth="1"/>
+    <col min="29" max="29" width="16" customWidth="1"/>
+    <col min="30" max="30" width="58" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -118,125 +119,130 @@
       </c>
       <c r="E1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Group Order</t>
+          <t xml:space="preserve">Passage Text</t>
         </is>
       </c>
       <c r="F1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Passage Text</t>
+          <t xml:space="preserve">Passage Image</t>
         </is>
       </c>
       <c r="G1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Passage Image</t>
+          <t xml:space="preserve">Question Text</t>
         </is>
       </c>
       <c r="H1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Question Text</t>
+          <t xml:space="preserve">Question Image</t>
         </is>
       </c>
       <c r="I1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Question Image</t>
+          <t xml:space="preserve">Question Type</t>
         </is>
       </c>
       <c r="J1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Question Type</t>
+          <t xml:space="preserve">Option A Text</t>
         </is>
       </c>
       <c r="K1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Option A Text</t>
+          <t xml:space="preserve">Option A Image</t>
         </is>
       </c>
       <c r="L1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Option A Image</t>
+          <t xml:space="preserve">Option B Text</t>
         </is>
       </c>
       <c r="M1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Option B Text</t>
+          <t xml:space="preserve">Option B Image</t>
         </is>
       </c>
       <c r="N1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Option B Image</t>
+          <t xml:space="preserve">Option C Text</t>
         </is>
       </c>
       <c r="O1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Option C Text</t>
+          <t xml:space="preserve">Option C Image</t>
         </is>
       </c>
       <c r="P1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Option C Image</t>
+          <t xml:space="preserve">Option D Text</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Option D Text</t>
+          <t xml:space="preserve">Option D Image</t>
         </is>
       </c>
       <c r="R1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Option D Image</t>
+          <t xml:space="preserve">Option E Text</t>
         </is>
       </c>
       <c r="S1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Option E Text</t>
+          <t xml:space="preserve">Option E Image</t>
         </is>
       </c>
       <c r="T1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Option E Image</t>
+          <t xml:space="preserve">Correct Option</t>
         </is>
       </c>
       <c r="U1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Correct Option</t>
+          <t xml:space="preserve">Explanation</t>
         </is>
       </c>
       <c r="V1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Explanation</t>
+          <t xml:space="preserve">Mode</t>
         </is>
       </c>
       <c r="W1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Mode</t>
+          <t xml:space="preserve">Active</t>
         </is>
       </c>
       <c r="X1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Active</t>
+          <t xml:space="preserve">Difficulty</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Difficulty</t>
+          <t xml:space="preserve">Marks</t>
         </is>
       </c>
       <c r="Z1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Marks</t>
+          <t xml:space="preserve">Negative Marks</t>
         </is>
       </c>
       <c r="AA1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Negative Marks</t>
+          <t xml:space="preserve">Scoring Rule</t>
         </is>
       </c>
       <c r="AB1" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">Shuffle Options</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">Ready For Import</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr" s="1">
+      <c r="AD1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Notes</t>
         </is>
@@ -274,11 +280,6 @@
         </is>
       </c>
       <c r="G2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
         <is>
           <t xml:space="preserve">Saira, Mumtaz and Zeenat have a ball, a pen and a pencil, and each girl has just one object in hand. Among the following statements, only one is true and the other two are false.
 I. Saira has a ball.
@@ -287,49 +288,54 @@
 Who has the ball?</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">single</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t xml:space="preserve">single</t>
+          <t xml:space="preserve">Saira</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Saira</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Mumtaz</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mumtaz</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Zeenat</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zeenat</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Cannot be determined</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cannot be determined</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -344,44 +350,49 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">B</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t xml:space="preserve">B</t>
+          <t xml:space="preserve">If Saira has the ball, statements I and II become true. If Zeenat has the ball, statements II and III become true. Only Mumtaz having the ball makes exactly one statement true.</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t xml:space="preserve">If Saira has the ball, statements I and II become true. If Zeenat has the ball, statements II and III become true. Only Mumtaz having the ball makes exactly one statement true.</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
           <t xml:space="preserve">demo</t>
         </is>
       </c>
-      <c r="X2">
-        <v>1</v>
-      </c>
-      <c r="Y2" t="inlineStr">
+      <c r="W2">
+        <v>1</v>
+      </c>
+      <c r="X2" t="inlineStr">
         <is>
           <t xml:space="preserve">medium</t>
         </is>
       </c>
+      <c r="Y2">
+        <v>1</v>
+      </c>
       <c r="Z2">
-        <v>1</v>
-      </c>
-      <c r="AA2">
         <v>0</v>
       </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact_match</t>
+        </is>
+      </c>
       <c r="AB2" t="inlineStr">
         <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AD2" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -420,57 +431,57 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Albert, David, Jerome and Tommy were plucking mangoes. Their earnings were directly related to the number of mangoes plucked. Jerome got less money than Tommy. Jerome and Tommy together got the same amount as Albert and David together. Albert and Tommy together got less than David and Jerome together. Who earned the most pocket money? Who plucked the least number of mangoes?</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Albert, David, Jerome and Tommy were plucking mangoes. Their earnings were directly related to the number of mangoes plucked. Jerome got less money than Tommy. Jerome and Tommy together got the same amount as Albert and David together. Albert and Tommy together got less than David and Jerome together. Who earned the most pocket money? Who plucked the least number of mangoes?</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">single</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t xml:space="preserve">single</t>
+          <t xml:space="preserve">David, Jerome</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t xml:space="preserve">David, Jerome</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">David, Albert</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t xml:space="preserve">David, Albert</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Jerome, Tommy</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jerome, Tommy</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Jerome, Albert</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jerome, Albert</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -485,44 +496,49 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">B</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t xml:space="preserve">B</t>
+          <t xml:space="preserve">Let earnings be A, D, J, T. Given J &lt; T and J + T = A + D. From A + T &lt; D + J and D = J + T - A, we get A &lt; J. Therefore A &lt; J &lt; T and D &gt; T, so David earned most and Albert least.</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Let earnings be A, D, J, T. Given J &lt; T and J + T = A + D. From A + T &lt; D + J and D = J + T - A, we get A &lt; J. Therefore A &lt; J &lt; T and D &gt; T, so David earned most and Albert least.</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
           <t xml:space="preserve">demo</t>
         </is>
       </c>
-      <c r="X3">
-        <v>1</v>
-      </c>
-      <c r="Y3" t="inlineStr">
+      <c r="W3">
+        <v>1</v>
+      </c>
+      <c r="X3" t="inlineStr">
         <is>
           <t xml:space="preserve">hard</t>
         </is>
       </c>
+      <c r="Y3">
+        <v>1</v>
+      </c>
       <c r="Z3">
-        <v>1</v>
-      </c>
-      <c r="AA3">
         <v>0</v>
       </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact_match</t>
+        </is>
+      </c>
       <c r="AB3" t="inlineStr">
         <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
-      <c r="AC3" t="inlineStr">
+      <c r="AD3" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -531,7 +547,7 @@
     <row r="4" ht="66" customHeight="1">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DI-RAIL-061</t>
+          <t xml:space="preserve">LR-MULTI-057</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -541,75 +557,77 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Data Interpretation</t>
+          <t xml:space="preserve">Number Classification</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DI-RAILWAY-COST-001</t>
-        </is>
-      </c>
-      <c r="E4">
-        <v>1</v>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve">The table/image below shows the estimated cost, in Rs. lakh, of a project for laying a railway line between two places. Keep the same passage/table reference repeated for every sub-question in this set.</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t xml:space="preserve">assets/question-media/railway-cost-estimate-table.png</t>
+          <t xml:space="preserve">Which of the following numbers are prime numbers? Select all correct options.</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t xml:space="preserve">The total expenditure is required to be kept within Rs. 700 lakh by cutting the expenditure on administration equally in all the years. What will be the percentage cut for 1989?</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">multi</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t xml:space="preserve">single</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t xml:space="preserve">22.6</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t xml:space="preserve">32.6</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">9</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t xml:space="preserve">42.5</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">11</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t xml:space="preserve">52.6</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -624,53 +642,58 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">A,B,D</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TBD</t>
+          <t xml:space="preserve">The numbers 2, 3, and 11 have exactly two positive factors. The number 9 is composite.</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fill after checking the railway cost table.</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">assessment</t>
-        </is>
-      </c>
-      <c r="X4">
-        <v>1</v>
-      </c>
-      <c r="Y4" t="inlineStr">
+          <t xml:space="preserve">demo</t>
+        </is>
+      </c>
+      <c r="W4">
+        <v>1</v>
+      </c>
+      <c r="X4" t="inlineStr">
         <is>
           <t xml:space="preserve">medium</t>
         </is>
       </c>
+      <c r="Y4">
+        <v>3</v>
+      </c>
       <c r="Z4">
         <v>1</v>
       </c>
-      <c r="AA4">
-        <v>0</v>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">partial_credit</t>
+        </is>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Grouped DI question. Keep same Group Code for all rows and use Group Order 1, 2, 3... so the group appears together in sequence. Correct option is marked TBD because the source table values were not included in the pasted text.</t>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partial-credit example: A,B,D earns 3 marks; selecting only A,B earns 2 marks; selecting any incorrect option such as C earns -1 mark.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="66" customHeight="1">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">DI-RAIL-062</t>
+          <t xml:space="preserve">IMG-SAMPLE-001</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -680,75 +703,77 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Data Interpretation</t>
+          <t xml:space="preserve">Visual Classification</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">DI-RAILWAY-COST-001</t>
-        </is>
-      </c>
-      <c r="E5">
-        <v>2</v>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t xml:space="preserve">The table/image below shows the estimated cost, in Rs. lakh, of a project for laying a railway line between two places. Keep the same passage/table reference repeated for every sub-question in this set.</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t xml:space="preserve">assets/question-media/railway-cost-estimate-table.png</t>
+          <t xml:space="preserve">The reference image shows the target color. Which option matches it?</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t xml:space="preserve">If the length of the line to be laid each year is proportional to the estimated cost for cement, steel, bricks, building material and labour, what fraction of the total length is proposed to be completed by the third year?</t>
+          <t xml:space="preserve">sample-color-guide.png</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">single</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t xml:space="preserve">single</t>
+          <t xml:space="preserve">Blue</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.9</t>
+          <t xml:space="preserve">blue-option.png</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Red</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.7</t>
+          <t xml:space="preserve">red-option.png</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Green</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.6</t>
+          <t xml:space="preserve">green-option.png</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Yellow</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.3</t>
+          <t xml:space="preserve">yellow-option.png</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -763,53 +788,58 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">A</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t xml:space="preserve">TBD</t>
+          <t xml:space="preserve">The reference image and option A both show blue.</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fill after checking the railway cost table.</t>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">assessment</t>
-        </is>
-      </c>
-      <c r="X5">
-        <v>1</v>
-      </c>
-      <c r="Y5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">medium</t>
-        </is>
+          <t xml:space="preserve">demo</t>
+        </is>
+      </c>
+      <c r="W5">
+        <v>1</v>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">easy</t>
+        </is>
+      </c>
+      <c r="Y5">
+        <v>1</v>
       </c>
       <c r="Z5">
-        <v>1</v>
-      </c>
-      <c r="AA5">
         <v>0</v>
       </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact_match</t>
+        </is>
+      </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Grouped DI question. Keep same Group Code for all rows and use Group Order 1, 2, 3... so the group appears together in sequence. Correct option is marked TBD because the source table values were not included in the pasted text.</t>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ready image example. Upload question_bank_sample_images.zip with the CSV; filenames may be inside any safe folders in the ZIP.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="66" customHeight="1">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">DI-RAIL-063</t>
+          <t xml:space="preserve">PASS-SOLAR-001-01</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -819,75 +849,77 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Data Interpretation</t>
+          <t xml:space="preserve">Passage Analysis</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">DI-RAILWAY-COST-001</t>
-        </is>
-      </c>
-      <c r="E6">
-        <v>3</v>
+          <t xml:space="preserve">PASS-SOLAR-001</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A school installed rooftop solar panels to reduce its electricity use. In April the panels generated 1,200 units of electricity, while the school consumed 1,500 units. In May generation increased by 25 percent from April, and consumption remained unchanged. Any generation beyond consumption is exported to the electricity grid.</t>
+        </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve">The table/image below shows the estimated cost, in Rs. lakh, of a project for laying a railway line between two places. Keep the same passage/table reference repeated for every sub-question in this set.</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t xml:space="preserve">assets/question-media/railway-cost-estimate-table.png</t>
+          <t xml:space="preserve">How many electricity units did the school obtain from the grid in April?</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t xml:space="preserve">What is the approximate ratio of the total cost of materials (cement, steel, bricks, building materials) for all the years to the total labour cost?</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">single</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t xml:space="preserve">single</t>
+          <t xml:space="preserve">200 units</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 : 1</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">300 units</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t xml:space="preserve">8 : 1</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">500 units</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t xml:space="preserve">12 : 1</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">1,200 units</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t xml:space="preserve">16 : 1</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -902,53 +934,58 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">B</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t xml:space="preserve">TBD</t>
+          <t xml:space="preserve">April consumption exceeded solar generation by 1,500 - 1,200 = 300 units.</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fill after checking the railway cost table.</t>
-        </is>
-      </c>
-      <c r="W6" t="inlineStr">
-        <is>
           <t xml:space="preserve">assessment</t>
         </is>
       </c>
-      <c r="X6">
-        <v>1</v>
-      </c>
-      <c r="Y6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">medium</t>
-        </is>
+      <c r="W6">
+        <v>1</v>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">easy</t>
+        </is>
+      </c>
+      <c r="Y6">
+        <v>1</v>
       </c>
       <c r="Z6">
-        <v>1</v>
-      </c>
-      <c r="AA6">
         <v>0</v>
       </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact_match</t>
+        </is>
+      </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Grouped DI question. Keep same Group Code for all rows and use Group Order 1, 2, 3... so the group appears together in sequence. Correct option is marked TBD because the source table values were not included in the pasted text.</t>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ready paragraph group. Keep all PASS-SOLAR-001 rows consecutive.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="66" customHeight="1">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">DI-RAIL-064</t>
+          <t xml:space="preserve">PASS-SOLAR-001-02</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -958,75 +995,77 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Data Interpretation</t>
+          <t xml:space="preserve">Passage Analysis</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">DI-RAILWAY-COST-001</t>
-        </is>
-      </c>
-      <c r="E7">
-        <v>4</v>
+          <t xml:space="preserve">PASS-SOLAR-001</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A school installed rooftop solar panels to reduce its electricity use. In April the panels generated 1,200 units of electricity, while the school consumed 1,500 units. In May generation increased by 25 percent from April, and consumption remained unchanged. Any generation beyond consumption is exported to the electricity grid.</t>
+        </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve">The table/image below shows the estimated cost, in Rs. lakh, of a project for laying a railway line between two places. Keep the same passage/table reference repeated for every sub-question in this set.</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t xml:space="preserve">assets/question-media/railway-cost-estimate-table.png</t>
+          <t xml:space="preserve">How many electricity units did the panels generate in May?</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t xml:space="preserve">If the cost of materials (cement, steel, bricks, building materials) rises by 5% each year from 1990 onwards, by how much will the estimated cost rise for the years 1990 and 1991?</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">single</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t xml:space="preserve">single</t>
+          <t xml:space="preserve">1,200 units</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rs. 11.45 lakh</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">1,350 units</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rs. 16.35 lakh</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">1,500 units</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rs. 21.45 lakh</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">1,800 units</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rs. 26.45 lakh</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1041,53 +1080,58 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">C</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t xml:space="preserve">TBD</t>
+          <t xml:space="preserve">A 25 percent increase on 1,200 units is 300 units, giving 1,500 units.</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fill after checking the railway cost table.</t>
-        </is>
-      </c>
-      <c r="W7" t="inlineStr">
-        <is>
           <t xml:space="preserve">assessment</t>
         </is>
       </c>
-      <c r="X7">
-        <v>1</v>
-      </c>
-      <c r="Y7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">medium</t>
-        </is>
+      <c r="W7">
+        <v>1</v>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">easy</t>
+        </is>
+      </c>
+      <c r="Y7">
+        <v>1</v>
       </c>
       <c r="Z7">
-        <v>1</v>
-      </c>
-      <c r="AA7">
         <v>0</v>
       </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact_match</t>
+        </is>
+      </c>
       <c r="AB7" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Grouped DI question. Keep same Group Code for all rows and use Group Order 1, 2, 3... so the group appears together in sequence. Correct option is marked TBD because the source table values were not included in the pasted text.</t>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ready paragraph group. Excel row order becomes protected group sequence.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="66" customHeight="1">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">DI-RAIL-065</t>
+          <t xml:space="preserve">PASS-SOLAR-001-03</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1097,75 +1141,77 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Data Interpretation</t>
+          <t xml:space="preserve">Passage Analysis</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">DI-RAILWAY-COST-001</t>
-        </is>
-      </c>
-      <c r="E8">
-        <v>5</v>
+          <t xml:space="preserve">PASS-SOLAR-001</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A school installed rooftop solar panels to reduce its electricity use. In April the panels generated 1,200 units of electricity, while the school consumed 1,500 units. In May generation increased by 25 percent from April, and consumption remained unchanged. Any generation beyond consumption is exported to the electricity grid.</t>
+        </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve">The table/image below shows the estimated cost, in Rs. lakh, of a project for laying a railway line between two places. Keep the same passage/table reference repeated for every sub-question in this set.</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t xml:space="preserve">assets/question-media/railway-cost-estimate-table.png</t>
+          <t xml:space="preserve">Which statements are correct for May? Select all correct options.</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t xml:space="preserve">It is found at the end of 1990 that the entire amount estimated for the project has been spent. If for 1991, the actual amount spent was equal to that which was estimated, by what percent (approximately) has the actual expenditure exceeded the estimated expenditure?</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">multi</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t xml:space="preserve">single</t>
+          <t xml:space="preserve">Solar generation equalled consumption.</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t xml:space="preserve">39</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">The school imported 300 units from the grid.</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t xml:space="preserve">29</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">No electricity was exported to the grid.</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t xml:space="preserve">19</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Generation was 25 percent higher than in April.</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t xml:space="preserve">9</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -1180,190 +1226,932 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">A,C,D</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t xml:space="preserve">TBD</t>
+          <t xml:space="preserve">May generation was 1,500 units, equal to consumption, so there was no import or export.</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fill after checking the railway cost table.</t>
-        </is>
-      </c>
-      <c r="W8" t="inlineStr">
-        <is>
           <t xml:space="preserve">assessment</t>
         </is>
       </c>
-      <c r="X8">
-        <v>1</v>
-      </c>
-      <c r="Y8" t="inlineStr">
+      <c r="W8">
+        <v>1</v>
+      </c>
+      <c r="X8" t="inlineStr">
         <is>
           <t xml:space="preserve">medium</t>
         </is>
       </c>
+      <c r="Y8">
+        <v>3</v>
+      </c>
       <c r="Z8">
         <v>1</v>
       </c>
-      <c r="AA8">
-        <v>0</v>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">partial_credit</t>
+        </is>
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t xml:space="preserve">No</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Grouped DI question. Keep same Group Code for all rows and use Group Order 1, 2, 3... so the group appears together in sequence. Correct option is marked TBD because the source table values were not included in the pasted text.</t>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ready multi-select member of the protected paragraph group.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="66" customHeight="1">
       <c r="A9" t="inlineStr">
         <is>
+          <t xml:space="preserve">DI-RAIL-061</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Logical Reasoning</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Data Interpretation</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DI-RAILWAY-COST-001</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The table/image below shows the estimated cost, in Rs. lakh, of a project for laying a railway line between two places. Keep the same passage/table reference repeated for every sub-question in this set.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">railway-cost-estimate-table.png</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The total expenditure is required to be kept within Rs. 700 lakh by cutting the expenditure on administration equally in all the years. What will be the percentage cut for 1989?</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">single</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">22.6</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">32.6</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">42.5</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">52.6</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TBD</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fill after checking the railway cost table.</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">assessment</t>
+        </is>
+      </c>
+      <c r="W9">
+        <v>1</v>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">medium</t>
+        </is>
+      </c>
+      <c r="Y9">
+        <v>1</v>
+      </c>
+      <c r="Z9">
+        <v>0</v>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact_match</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Grouped DI question. Keep the same Group Code and keep all group rows consecutive. Their Excel row order becomes the protected sequence. Correct option is marked TBD because the source table values were not included in the pasted text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="66" customHeight="1">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DI-RAIL-062</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Logical Reasoning</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Data Interpretation</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DI-RAILWAY-COST-001</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The table/image below shows the estimated cost, in Rs. lakh, of a project for laying a railway line between two places. Keep the same passage/table reference repeated for every sub-question in this set.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">railway-cost-estimate-table.png</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">If the length of the line to be laid each year is proportional to the estimated cost for cement, steel, bricks, building material and labour, what fraction of the total length is proposed to be completed by the third year?</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">single</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.9</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.7</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.6</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.3</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TBD</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fill after checking the railway cost table.</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">assessment</t>
+        </is>
+      </c>
+      <c r="W10">
+        <v>1</v>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">medium</t>
+        </is>
+      </c>
+      <c r="Y10">
+        <v>1</v>
+      </c>
+      <c r="Z10">
+        <v>0</v>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact_match</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Grouped DI question. Keep the same Group Code and keep all group rows consecutive. Their Excel row order becomes the protected sequence. Correct option is marked TBD because the source table values were not included in the pasted text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="66" customHeight="1">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DI-RAIL-063</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Logical Reasoning</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Data Interpretation</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DI-RAILWAY-COST-001</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The table/image below shows the estimated cost, in Rs. lakh, of a project for laying a railway line between two places. Keep the same passage/table reference repeated for every sub-question in this set.</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">railway-cost-estimate-table.png</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">What is the approximate ratio of the total cost of materials (cement, steel, bricks, building materials) for all the years to the total labour cost?</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">single</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 : 1</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8 : 1</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12 : 1</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16 : 1</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TBD</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fill after checking the railway cost table.</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">assessment</t>
+        </is>
+      </c>
+      <c r="W11">
+        <v>1</v>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">medium</t>
+        </is>
+      </c>
+      <c r="Y11">
+        <v>1</v>
+      </c>
+      <c r="Z11">
+        <v>0</v>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact_match</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Grouped DI question. Keep the same Group Code and keep all group rows consecutive. Their Excel row order becomes the protected sequence. Correct option is marked TBD because the source table values were not included in the pasted text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="66" customHeight="1">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DI-RAIL-064</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Logical Reasoning</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Data Interpretation</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DI-RAILWAY-COST-001</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The table/image below shows the estimated cost, in Rs. lakh, of a project for laying a railway line between two places. Keep the same passage/table reference repeated for every sub-question in this set.</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">railway-cost-estimate-table.png</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">If the cost of materials (cement, steel, bricks, building materials) rises by 5% each year from 1990 onwards, by how much will the estimated cost rise for the years 1990 and 1991?</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">single</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rs. 11.45 lakh</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rs. 16.35 lakh</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rs. 21.45 lakh</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rs. 26.45 lakh</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TBD</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fill after checking the railway cost table.</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">assessment</t>
+        </is>
+      </c>
+      <c r="W12">
+        <v>1</v>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">medium</t>
+        </is>
+      </c>
+      <c r="Y12">
+        <v>1</v>
+      </c>
+      <c r="Z12">
+        <v>0</v>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact_match</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Grouped DI question. Keep the same Group Code and keep all group rows consecutive. Their Excel row order becomes the protected sequence. Correct option is marked TBD because the source table values were not included in the pasted text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="66" customHeight="1">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DI-RAIL-065</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Logical Reasoning</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Data Interpretation</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DI-RAILWAY-COST-001</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The table/image below shows the estimated cost, in Rs. lakh, of a project for laying a railway line between two places. Keep the same passage/table reference repeated for every sub-question in this set.</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">railway-cost-estimate-table.png</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">It is found at the end of 1990 that the entire amount estimated for the project has been spent. If for 1991, the actual amount spent was equal to that which was estimated, by what percent (approximately) has the actual expenditure exceeded the estimated expenditure?</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">single</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">39</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">29</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">19</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TBD</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fill after checking the railway cost table.</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">assessment</t>
+        </is>
+      </c>
+      <c r="W13">
+        <v>1</v>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">medium</t>
+        </is>
+      </c>
+      <c r="Y13">
+        <v>1</v>
+      </c>
+      <c r="Z13">
+        <v>0</v>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact_match</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Grouped DI question. Keep the same Group Code and keep all group rows consecutive. Their Excel row order becomes the protected sequence. Correct option is marked TBD because the source table values were not included in the pasted text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="66" customHeight="1">
+      <c r="A14" t="inlineStr">
+        <is>
           <t xml:space="preserve">DI-RAIL-066</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t xml:space="preserve">Logical Reasoning</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t xml:space="preserve">Data Interpretation</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t xml:space="preserve">DI-RAILWAY-COST-001</t>
         </is>
       </c>
-      <c r="E9">
-        <v>6</v>
-      </c>
-      <c r="F9" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t xml:space="preserve">The table/image below shows the estimated cost, in Rs. lakh, of a project for laying a railway line between two places. Keep the same passage/table reference repeated for every sub-question in this set.</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">assets/question-media/railway-cost-estimate-table.png</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
+      <c r="F14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">railway-cost-estimate-table.png</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
         <is>
           <t xml:space="preserve">After preparing the estimate, the provision for contingencies is felt inadequate and is therefore doubled. By what percent does the total estimate increase?</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
+      <c r="H14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
         <is>
           <t xml:space="preserve">single</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t xml:space="preserve">3.47</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
+      <c r="K14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
         <is>
           <t xml:space="preserve">2.45</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
+      <c r="M14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
         <is>
           <t xml:space="preserve">1.50</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
+      <c r="O14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
         <is>
           <t xml:space="preserve">3.62</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="T9" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
         <is>
           <t xml:space="preserve">TBD</t>
         </is>
       </c>
-      <c r="V9" t="inlineStr">
+      <c r="U14" t="inlineStr">
         <is>
           <t xml:space="preserve">Fill after checking the railway cost table.</t>
         </is>
       </c>
-      <c r="W9" t="inlineStr">
+      <c r="V14" t="inlineStr">
         <is>
           <t xml:space="preserve">assessment</t>
         </is>
       </c>
-      <c r="X9">
-        <v>1</v>
-      </c>
-      <c r="Y9" t="inlineStr">
+      <c r="W14">
+        <v>1</v>
+      </c>
+      <c r="X14" t="inlineStr">
         <is>
           <t xml:space="preserve">medium</t>
         </is>
       </c>
-      <c r="Z9">
-        <v>1</v>
-      </c>
-      <c r="AA9">
+      <c r="Y14">
+        <v>1</v>
+      </c>
+      <c r="Z14">
         <v>0</v>
       </c>
-      <c r="AB9" t="inlineStr">
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact_match</t>
+        </is>
+      </c>
+      <c r="AB14" t="inlineStr">
         <is>
           <t xml:space="preserve">No</t>
         </is>
       </c>
-      <c r="AC9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Grouped DI question. Keep same Group Code for all rows and use Group Order 1, 2, 3... so the group appears together in sequence. Correct option is marked TBD because the source table values were not included in the pasted text.</t>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Grouped DI question. Keep the same Group Code and keep all group rows consecutive. Their Excel row order becomes the protected sequence. Correct option is marked TBD because the source table values were not included in the pasted text.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AC9"/>
+  <autoFilter ref="A1:AD14"/>
 </worksheet>
 </file>
 
@@ -1413,12 +2201,12 @@
     <row r="4" ht="66" customHeight="1">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Group Order</t>
+          <t xml:space="preserve">Group Sequence</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Blank for standalone questions. Use 1, 2, 3... inside a grouped set.</t>
+          <t xml:space="preserve">There is no order column. Keep group rows consecutive; Excel row order becomes their protected sequence.</t>
         </is>
       </c>
     </row>
@@ -1442,7 +2230,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use when the question depends on a table/diagram image. Example: assets/question-media/railway-cost-estimate-table.png</t>
+          <t xml:space="preserve">Enter the matching ZIP filename, such as railway-cost-estimate-table.png.</t>
         </is>
       </c>
     </row>
@@ -1485,28 +2273,112 @@
     <row r="10" ht="66" customHeight="1">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ready For Import</t>
+          <t xml:space="preserve">Marks</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use Yes only after correct option, media path, and explanation are final.</t>
+          <t xml:space="preserve">Positive marks awarded when the answer satisfies the scoring rule.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="66" customHeight="1">
       <c r="A11" t="inlineStr">
         <is>
+          <t xml:space="preserve">Negative Marks</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Deduction applied to an answered response that includes a wrong option or fails exact_match.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="66" customHeight="1">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scoring Rule</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Use exact_match or partial_credit. Blank defaults to exact_match.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="66" customHeight="1">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exact_match</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Full marks only when the selected set exactly matches Correct Option; otherwise deduct Negative Marks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="66" customHeight="1">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">partial_credit</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A correct subset with no wrong option earns proportional marks; any wrong selected option deducts Negative Marks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="66" customHeight="1">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shuffle Options</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Use Yes to randomize option order once per attempt, or No to keep A, B, C order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="66" customHeight="1">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ready For Import</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Use Yes only after correct option, media path, and explanation are final.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="66" customHeight="1">
+      <c r="A17" t="inlineStr">
+        <is>
           <t xml:space="preserve">Randomization Rule</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Randomize standalone questions and group placement. Once a group starts, display its rows by Group Order.</t>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standalone questions and complete groups may shuffle. Questions inside a group stay in consecutive Excel row order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="66" customHeight="1">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Image ZIP</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZIP image names must match workbook image cells. The importer validates, converts to WebP, and creates a unique server batch folder.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B11"/>
+  <autoFilter ref="A1:B18"/>
 </worksheet>
 </file>
</xml_diff>